<commit_message>
feat: clean transactions (closed, refunds, partial refunds, duplicates)
- core/clean.py: rules with removal reasons; totals() ignores neutral records
- import page shows cleaned totals and an expander listing removed records
- fixtures: add partial refund and refund-income rows

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/wechat_sample.xlsx
+++ b/tests/fixtures/wechat_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,21 +454,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>共5笔记录</t>
+          <t>共7笔记录</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>收入：1笔 ¥52.00</t>
+          <t>收入：2笔 ¥82.00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>支出：3笔 ¥73.80</t>
+          <t>支出：4笔 ¥153.80</t>
         </is>
       </c>
     </row>
@@ -844,6 +844,120 @@
         </is>
       </c>
       <c r="K21" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-12 15:40:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>商户消费</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>拼多多商家</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>T恤 两件</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>支出</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>¥80.00</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>零钱</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>已退款(¥30.00)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>4200002026091200006</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>PD20260912006</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>拼多多商家-退款</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>拼多多商家</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>收入</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>¥30.00</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>零钱</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>已退款</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>4200002026091400007</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>PD20260912006</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>/</t>
         </is>

</xml_diff>

<commit_message>
feat: count cross-month refunds as negative spending (product decision Q1)
Refund records are matched to their original order by total refunded amount
(the refund status carries it, e.g. 已退款¥131.50). Unmatched refunds become
negative spending in the current period.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/wechat_sample.xlsx
+++ b/tests/fixtures/wechat_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,14 +454,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>共7笔记录</t>
+          <t>共8笔记录</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>收入：2笔 ¥82.00</t>
+          <t>收入：3笔 ¥127.00</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>已退款</t>
+          <t>已退款¥30.00</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -954,10 +954,67 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>PD20260912006</t>
+          <t>/</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-08 11:20:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>中铁网络-退款</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>中铁网络</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>收入</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>¥45.00</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>零钱</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>已全额退款</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>4200002026090800008</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>/</t>
         </is>

</xml_diff>